<commit_message>
Update edition crosswalk release status
</commit_message>
<xml_diff>
--- a/docs/architecture/AI_Playbook_Edition_Crosswalk.xlsx
+++ b/docs/architecture/AI_Playbook_Edition_Crosswalk.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R67a91c01cb184045"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Crosswalk" sheetId="2" r:id="R8503debb75ae4592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Crosswalk" sheetId="3" r:id="R9b52e455b1c9426c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="4" r:id="Rdf5280da264542a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="5" r:id="Rfb5adccb39aa47e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R3e1f7580f4ee4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R724c1a83d40141e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Crosswalk" sheetId="2" r:id="R22203718834b49e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Crosswalk" sheetId="3" r:id="R3870c11effb045f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="4" r:id="R7bc0d46db62140e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="5" r:id="R0e8592719763468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="6" r:id="R17da31b5fa6049bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -136,7 +136,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -257,6 +257,18 @@
     <x:xf numFmtId="200" fontId="8" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -268,7 +280,7 @@
         <x:color rgb="FF9C1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -279,7 +291,7 @@
         <x:color rgb="FF368F2C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDF8EE"/>
         </x:patternFill>
       </x:fill>
@@ -289,8 +301,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureCrosswalk" displayName="FeatureCrosswalk" ref="A4:R47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:R47"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureCrosswalk" displayName="FeatureCrosswalk" ref="A4:R48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:R48"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="Stable ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -356,8 +368,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ChangeLog" displayName="ChangeLog" ref="A4:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ChangeLog" displayName="ChangeLog" ref="A4:L10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L10"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Change ID"/>
     <x:tableColumn id="2" name="Stable Item ID"/>
@@ -607,7 +619,7 @@
         <x:v>Workbook version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>Tracked features</x:v>
@@ -634,19 +646,19 @@
       </x:c>
       <x:c r="D6" s="23" t="n">
         <x:f>COUNTA('Feature Crosswalk'!A5:A204)</x:f>
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF('Feature Crosswalk'!H5:H204,"Yes")</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F6" s="23" t="n">
         <x:f>COUNTIF('Feature Crosswalk'!L5:L204,"In Progress")</x:f>
-        <x:v>19</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="23" t="n">
         <x:f>COUNTIF('Feature Crosswalk'!L5:L204,"Complete")</x:f>
-        <x:v>11</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H6" s="23" t="n">
         <x:f>COUNTIF('Feature Crosswalk'!M5:M204,"TBD")</x:f>
@@ -1006,27 +1018,29 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="G6" s="47" t="str">
-        <x:v>Shared template system added locally; requires final regression review</x:v>
+        <x:v>Shared template system released for both editions</x:v>
       </x:c>
       <x:c r="H6" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I6" s="50" t="str">
-        <x:v>Confirm every Full and Foundation page type uses shared templates and responsive rules</x:v>
+        <x:v>Maintain one shared template layer and regression-test both edition destinations</x:v>
       </x:c>
       <x:c r="J6" s="50" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="K6" s="50" t="str"/>
       <x:c r="L6" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="M6" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="N6" s="56" t="str"/>
+      <x:c r="N6" s="56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
       <x:c r="O6" s="56" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="P6" s="47" t="str"/>
       <x:c r="Q6" s="47" t="str"/>
@@ -1108,27 +1122,29 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G8" s="47" t="str">
-        <x:v>Foundation lacks organization-level access</x:v>
+        <x:v>Shared navigation definition released with intentional entitlement differences</x:v>
       </x:c>
       <x:c r="H8" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I8" s="50" t="str">
-        <x:v>Maintain one navigation definition with edition-aware destinations and entitlements</x:v>
+        <x:v>Keep labels and order aligned; Organization Hub remains an organization-level benefit</x:v>
       </x:c>
       <x:c r="J8" s="50" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="K8" s="50" t="str"/>
       <x:c r="L8" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="M8" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="N8" s="56" t="str"/>
+      <x:c r="N8" s="56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
       <x:c r="O8" s="56" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="P8" s="47" t="str"/>
       <x:c r="Q8" s="47" t="str"/>
@@ -1204,27 +1220,29 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G10" s="47" t="str">
-        <x:v>Content and buttons differ by edition; layout should match</x:v>
+        <x:v>Shared homepage structure released with edition-specific content and buttons</x:v>
       </x:c>
       <x:c r="H10" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I10" s="50" t="str">
-        <x:v>Use same dimensions, typography, spacing, journey image, and hotspots</x:v>
+        <x:v>Retain shared dimensions, typography, spacing, journey image, and edition-local hotspots</x:v>
       </x:c>
       <x:c r="J10" s="50" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="K10" s="50" t="str"/>
       <x:c r="L10" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="M10" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="N10" s="56" t="str"/>
+      <x:c r="N10" s="56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
       <x:c r="O10" s="56" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="P10" s="47" t="str">
         <x:v>#/</x:v>
@@ -1310,27 +1328,29 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G12" s="47" t="str">
-        <x:v>Counts and availability differ</x:v>
+        <x:v>Concise balanced overview released in both editions</x:v>
       </x:c>
       <x:c r="H12" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I12" s="50" t="str">
-        <x:v>Preserve equal emphasis on plays, tools, and learning</x:v>
+        <x:v>Preserve equal emphasis on plays, tools, and learning while retaining edition-specific counts</x:v>
       </x:c>
       <x:c r="J12" s="50" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="K12" s="50" t="str"/>
       <x:c r="L12" s="50" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="M12" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="N12" s="56" t="str"/>
+      <x:c r="N12" s="56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
       <x:c r="O12" s="56" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="P12" s="47" t="str"/>
       <x:c r="Q12" s="47" t="str"/>
@@ -1358,27 +1378,29 @@
         <x:v>Foundation Only</x:v>
       </x:c>
       <x:c r="G13" s="47" t="str">
-        <x:v>Commercial positioning belongs primarily in Foundation</x:v>
+        <x:v>Foundation comparison now distinguishes entry access from organization and enterprise editions</x:v>
       </x:c>
       <x:c r="H13" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I13" s="50" t="str">
-        <x:v>State what is available now, membership benefits, and future edition capabilities without implying unfinished content</x:v>
+        <x:v>Keep availability language current without implying completed content is unfinished</x:v>
       </x:c>
       <x:c r="J13" s="50" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="K13" s="50" t="str"/>
       <x:c r="L13" s="50" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="M13" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="N13" s="56" t="str"/>
+      <x:c r="N13" s="56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
       <x:c r="O13" s="56" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="P13" s="47" t="str"/>
       <x:c r="Q13" s="47" t="str"/>
@@ -3056,16 +3078,59 @@
         <x:v>46255.666666666664</x:v>
       </x:c>
     </x:row>
-    <x:row r="48">
-      <x:c r="H48" s="15"/>
-      <x:c r="I48" s="15"/>
-      <x:c r="J48" s="15"/>
-      <x:c r="K48" s="15"/>
-      <x:c r="L48" s="15"/>
-      <x:c r="M48" s="15"/>
-      <x:c r="N48" s="15"/>
-      <x:c r="O48" s="15"/>
-      <x:c r="R48" s="15"/>
+    <x:row r="48" ht="42" customHeight="1">
+      <x:c r="A48" s="58" t="str">
+        <x:v>PLAT-006</x:v>
+      </x:c>
+      <x:c r="B48" s="58" t="str">
+        <x:v>Shared platform</x:v>
+      </x:c>
+      <x:c r="C48" s="58" t="str">
+        <x:v>Inline code documentation</x:v>
+      </x:c>
+      <x:c r="D48" s="58" t="str">
+        <x:v>File-level contracts, schemas, business rules, persistence, accessibility, and maintenance guidance</x:v>
+      </x:c>
+      <x:c r="E48" s="58" t="str">
+        <x:v>Edition boundaries, local routing, account prototypes, learning assessment, and tool behavior documented</x:v>
+      </x:c>
+      <x:c r="F48" s="58" t="str">
+        <x:v>Same</x:v>
+      </x:c>
+      <x:c r="G48" s="58" t="str">
+        <x:v>Documentation explains shared rules and intentional edition differences</x:v>
+      </x:c>
+      <x:c r="H48" s="59" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I48" s="59" t="str">
+        <x:v>Update documentation in the same commit whenever a contract, schema, route, or business rule changes</x:v>
+      </x:c>
+      <x:c r="J48" s="59" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K48" s="59"/>
+      <x:c r="L48" s="59" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="M48" s="60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="N48" s="60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="O48" s="60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="P48" s="58" t="str">
+        <x:v>app.js; content/</x:v>
+      </x:c>
+      <x:c r="Q48" s="58" t="str">
+        <x:v>mvp/</x:v>
+      </x:c>
+      <x:c r="R48" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="H49" s="15"/>
@@ -3116,7 +3181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb72e601490fc49e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6a748284c6f4088"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3224,16 +3289,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J5" s="49" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K5" s="49" t="str">
-        <x:v>Finish shared-template regression review</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L5" s="55" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M5" s="49" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N5" s="52" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3532,16 +3597,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J12" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K12" s="50" t="str">
-        <x:v>Keep sequence and titles aligned</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L12" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M12" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N12" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3576,16 +3641,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J13" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K13" s="50" t="str">
-        <x:v>Use shared detail template</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L13" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M13" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N13" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3664,16 +3729,16 @@
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="J15" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K15" s="50" t="str">
-        <x:v>Standardize common shell and intro</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L15" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M15" s="50" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N15" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3752,16 +3817,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J17" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K17" s="50" t="str">
-        <x:v>Clarify administrator view and simplify</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L17" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M17" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N17" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3840,16 +3905,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J19" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K19" s="50" t="str">
-        <x:v>Remove edition marketing from this page</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L19" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M19" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N19" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3884,16 +3949,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J20" s="50" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K20" s="50" t="str">
-        <x:v>No tool contribution solicitation</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L20" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M20" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N20" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -3972,16 +4037,16 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="J22" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K22" s="50" t="str">
-        <x:v>Common provenance and review metadata</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L22" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M22" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N22" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -4016,16 +4081,16 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="J23" s="50" t="str">
-        <x:v>Review</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="K23" s="50" t="str">
-        <x:v>Automated ingestion still needs production service</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L23" s="56" t="str">
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="M23" s="50" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="N23" s="53" t="n">
         <x:v>46255.666666666664</x:v>
@@ -4063,7 +4128,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="K24" s="51" t="str">
-        <x:v>Keep content synchronized</x:v>
+        <x:v>Shared template/content change approved and released; continue regression review with future edits</x:v>
       </x:c>
       <x:c r="L24" s="57" t="str">
         <x:v>0.9</x:v>
@@ -4275,7 +4340,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8bf6a187bcc4e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re59ee2c4c55a4a31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6214,7 +6279,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca4b808f95e4b28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b3e99d875df4200"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6285,7 +6350,7 @@
         <x:v>Validation Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="49" t="str">
         <x:v>CHG-0001</x:v>
       </x:c>
@@ -6311,15 +6376,19 @@
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="I5" s="49" t="str">
-        <x:v>In Progress</x:v>
-      </x:c>
-      <x:c r="J5" s="52" t="str"/>
-      <x:c r="K5" s="49" t="str"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J5" s="52" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K5" s="49" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
       <x:c r="L5" s="49" t="str">
-        <x:v>Shared template layer added locally; regression validation pending</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+        <x:v>Shared template layer released; syntax and formatting checks passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="50" t="str">
         <x:v>CHG-0002</x:v>
       </x:c>
@@ -6345,15 +6414,19 @@
         <x:v>1.0</x:v>
       </x:c>
       <x:c r="I6" s="50" t="str">
-        <x:v>In Progress</x:v>
-      </x:c>
-      <x:c r="J6" s="53" t="str"/>
-      <x:c r="K6" s="50" t="str"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J6" s="53" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K6" s="50" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
       <x:c r="L6" s="50" t="str">
-        <x:v>Foundation comparison content added locally</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>Foundation edition comparison and concise overview released</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="51" t="str">
         <x:v>CHG-0003</x:v>
       </x:c>
@@ -6384,52 +6457,126 @@
       <x:c r="J7" s="54" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
-      <x:c r="K7" s="51" t="str"/>
+      <x:c r="K7" s="51" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
       <x:c r="L7" s="51" t="str">
-        <x:v>Workbook created</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="15"/>
-      <x:c r="B8" s="15"/>
-      <x:c r="C8" s="15"/>
-      <x:c r="D8" s="15"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
-      <x:c r="G8" s="14"/>
-      <x:c r="H8" s="13"/>
-      <x:c r="I8" s="15"/>
-      <x:c r="J8" s="14"/>
-      <x:c r="K8" s="15"/>
-      <x:c r="L8" s="15"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="15"/>
-      <x:c r="B9" s="15"/>
-      <x:c r="C9" s="15"/>
-      <x:c r="D9" s="15"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="14"/>
-      <x:c r="H9" s="13"/>
-      <x:c r="I9" s="15"/>
-      <x:c r="J9" s="14"/>
-      <x:c r="K9" s="15"/>
-      <x:c r="L9" s="15"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="15"/>
-      <x:c r="B10" s="15"/>
-      <x:c r="C10" s="15"/>
-      <x:c r="D10" s="15"/>
-      <x:c r="E10" s="15"/>
-      <x:c r="F10" s="15"/>
-      <x:c r="G10" s="14"/>
-      <x:c r="H10" s="13"/>
-      <x:c r="I10" s="15"/>
-      <x:c r="J10" s="14"/>
-      <x:c r="K10" s="15"/>
-      <x:c r="L10" s="15"/>
+        <x:v>Workbook published in repository and updated for release control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="59" t="str">
+        <x:v>CHG-0004</x:v>
+      </x:c>
+      <x:c r="B8" s="59" t="str">
+        <x:v>PLAT-006</x:v>
+      </x:c>
+      <x:c r="C8" s="59" t="str">
+        <x:v>Add meticulous inline documentation for application contracts and business rules</x:v>
+      </x:c>
+      <x:c r="D8" s="59" t="str">
+        <x:v>Maintainability and release-safety review</x:v>
+      </x:c>
+      <x:c r="E8" s="59" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="F8" s="59" t="str">
+        <x:v>Paula Soper</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="H8" s="60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="I8" s="59" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J8" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K8" s="59" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
+      <x:c r="L8" s="59" t="str">
+        <x:v>All 38 JavaScript files passed syntax validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="59" t="str">
+        <x:v>CHG-0005</x:v>
+      </x:c>
+      <x:c r="B9" s="59" t="str">
+        <x:v>CONSULT-001</x:v>
+      </x:c>
+      <x:c r="C9" s="59" t="str">
+        <x:v>Make consulting support more obvious in both editions</x:v>
+      </x:c>
+      <x:c r="D9" s="59" t="str">
+        <x:v>Customer pathway review</x:v>
+      </x:c>
+      <x:c r="E9" s="59" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="F9" s="59" t="str">
+        <x:v>Paula Soper</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="H9" s="60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="I9" s="59" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J9" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K9" s="59" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
+      <x:c r="L9" s="59" t="str">
+        <x:v>Shared navigation includes Consulting Support; edition-local destinations retained</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="59" t="str">
+        <x:v>CHG-0006</x:v>
+      </x:c>
+      <x:c r="B10" s="59" t="str">
+        <x:v>GOV-001</x:v>
+      </x:c>
+      <x:c r="C10" s="59" t="str">
+        <x:v>Refresh edition crosswalk after approved text, template, and documentation release</x:v>
+      </x:c>
+      <x:c r="D10" s="59" t="str">
+        <x:v>Release-control update</x:v>
+      </x:c>
+      <x:c r="E10" s="59" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="F10" s="59" t="str">
+        <x:v>Paula Soper</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="H10" s="60" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="I10" s="59" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="J10" s="61" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K10" s="59" t="str">
+        <x:v>17dea89</x:v>
+      </x:c>
+      <x:c r="L10" s="59" t="str">
+        <x:v>Statuses, version fields, routes, and audit log reconciled with GitHub main</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="15"/>
@@ -7773,7 +7920,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafecc3d2f1bf4366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d5bf8c4267545f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Rename Foundation Edition to Essentials Edition
</commit_message>
<xml_diff>
--- a/docs/architecture/AI_Playbook_Edition_Crosswalk.xlsx
+++ b/docs/architecture/AI_Playbook_Edition_Crosswalk.xlsx
@@ -308,7 +308,7 @@
     <x:tableColumn id="2" name="Area"/>
     <x:tableColumn id="3" name="Capability / Content"/>
     <x:tableColumn id="4" name="Full Version"/>
-    <x:tableColumn id="5" name="Foundation Version"/>
+    <x:tableColumn id="5" name="Essentials Version"/>
     <x:tableColumn id="6" name="Parity Status"/>
     <x:tableColumn id="7" name="Difference / Rationale"/>
     <x:tableColumn id="8" name="Change Needed"/>
@@ -320,7 +320,7 @@
     <x:tableColumn id="14" name="First Released Version"/>
     <x:tableColumn id="15" name="Last Changed Version"/>
     <x:tableColumn id="16" name="Full Route / Source"/>
-    <x:tableColumn id="17" name="Foundation Route / Source"/>
+    <x:tableColumn id="17" name="Essentials Route / Source"/>
     <x:tableColumn id="18" name="Last Reviewed"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -334,10 +334,10 @@
     <x:tableColumn id="1" name="Page ID"/>
     <x:tableColumn id="2" name="Navigation / Page"/>
     <x:tableColumn id="3" name="Full Version Route"/>
-    <x:tableColumn id="4" name="Foundation Route"/>
+    <x:tableColumn id="4" name="Essentials Route"/>
     <x:tableColumn id="5" name="Shared Template Type"/>
     <x:tableColumn id="6" name="Full Content Scope"/>
-    <x:tableColumn id="7" name="Foundation Content Scope"/>
+    <x:tableColumn id="7" name="Essentials Content Scope"/>
     <x:tableColumn id="8" name="Access Difference"/>
     <x:tableColumn id="9" name="Parity Status"/>
     <x:tableColumn id="10" name="Change Needed"/>
@@ -359,8 +359,8 @@
     <x:tableColumn id="3" name="Canonical Number / Code"/>
     <x:tableColumn id="4" name="Canonical Title"/>
     <x:tableColumn id="5" name="Full Version Availability"/>
-    <x:tableColumn id="6" name="Foundation Availability"/>
-    <x:tableColumn id="7" name="Foundation Mapping / Notes"/>
+    <x:tableColumn id="6" name="Essentials Availability"/>
+    <x:tableColumn id="7" name="Essentials Mapping / Notes"/>
     <x:tableColumn id="8" name="Target / Release Version"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -600,7 +600,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Release-control workbook for comparing the Full Version and Foundation Edition. Yellow cells are intended for future updates.</x:v>
+        <x:v>Release-control workbook for comparing the Full Version and Essentials Edition. Yellow cells are intended for future updates.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -675,10 +675,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="12" t="str">
-        <x:v>Foundation product name</x:v>
+        <x:v>Essentials product name</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>AI Playbook and Toolkit — Foundation Edition</x:v>
+        <x:v>AI Playbook and Toolkit — Essentials Edition</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -734,7 +734,7 @@
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="F21" s="34" t="str">
-        <x:v>Foundation intentionally exposes a smaller subset</x:v>
+        <x:v>Essentials intentionally exposes a smaller subset</x:v>
       </x:c>
       <x:c r="G21" s="34" t="str">
         <x:v>Not Available</x:v>
@@ -771,7 +771,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="35" t="str">
-        <x:v>Current Foundation baseline</x:v>
+        <x:v>Current Essentials baseline</x:v>
       </x:c>
       <x:c r="B23" s="35" t="str">
         <x:v>0.9</x:v>
@@ -886,7 +886,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Full vs Foundation — Feature Crosswalk</x:v>
+        <x:v>Full vs Essentials — Feature Crosswalk</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
@@ -908,7 +908,7 @@
         <x:v>Full Version</x:v>
       </x:c>
       <x:c r="E4" s="38" t="str">
-        <x:v>Foundation Version</x:v>
+        <x:v>Essentials Version</x:v>
       </x:c>
       <x:c r="F4" s="38" t="str">
         <x:v>Parity Status</x:v>
@@ -944,7 +944,7 @@
         <x:v>Full Route / Source</x:v>
       </x:c>
       <x:c r="Q4" s="38" t="str">
-        <x:v>Foundation Route / Source</x:v>
+        <x:v>Essentials Route / Source</x:v>
       </x:c>
       <x:c r="R4" s="38" t="str">
         <x:v>Last Reviewed</x:v>
@@ -970,7 +970,7 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G5" s="46" t="str">
-        <x:v>Foundation exposes a controlled subset while retaining canonical IDs</x:v>
+        <x:v>Essentials exposes a controlled subset while retaining canonical IDs</x:v>
       </x:c>
       <x:c r="H5" s="49" t="str">
         <x:v>Review</x:v>
@@ -1214,7 +1214,7 @@
         <x:v>Full positioning and Full-specific calls to action</x:v>
       </x:c>
       <x:c r="E10" s="47" t="str">
-        <x:v>Same template with Foundation positioning and Foundation destinations</x:v>
+        <x:v>Same template with Essentials positioning and Essentials destinations</x:v>
       </x:c>
       <x:c r="F10" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -1268,7 +1268,7 @@
         <x:v>Canonical journey graphic; links to Full assessment and phase sections</x:v>
       </x:c>
       <x:c r="E11" s="47" t="str">
-        <x:v>Same image; links remain within Foundation</x:v>
+        <x:v>Same image; links remain within Essentials</x:v>
       </x:c>
       <x:c r="F11" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -1322,7 +1322,7 @@
         <x:v>Concise overview of playbook, 49 tools, and 89-module learning catalog</x:v>
       </x:c>
       <x:c r="E12" s="47" t="str">
-        <x:v>Concise overview of playbook, 13 Foundation Tools, and Foundation learning</x:v>
+        <x:v>Concise overview of playbook, 13 Essentials Tools, and Essentials learning</x:v>
       </x:c>
       <x:c r="F12" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -1372,13 +1372,13 @@
         <x:v>Full site presents complete capabilities</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Foundation explains free/low-cost entry point and forthcoming robust editions</x:v>
+        <x:v>Essentials explains free/low-cost entry point and forthcoming robust editions</x:v>
       </x:c>
       <x:c r="F13" s="47" t="str">
-        <x:v>Foundation Only</x:v>
+        <x:v>Essentials Only</x:v>
       </x:c>
       <x:c r="G13" s="47" t="str">
-        <x:v>Foundation comparison now distinguishes entry access from organization and enterprise editions</x:v>
+        <x:v>Essentials comparison now distinguishes entry access from organization and enterprise editions</x:v>
       </x:c>
       <x:c r="H13" s="50" t="str">
         <x:v>No</x:v>
@@ -1422,7 +1422,7 @@
         <x:v>Available; generates scored readiness results and recommended plays/tools</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Available with free account prerequisite; saves results and generates Foundation destinations</x:v>
+        <x:v>Available with free account prerequisite; saves results and generates Essentials destinations</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -1474,13 +1474,13 @@
         <x:v>Recommends plays and Full tools in numeric/dependency order</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Recommends plays and available Foundation Tools</x:v>
+        <x:v>Recommends plays and available Essentials Tools</x:v>
       </x:c>
       <x:c r="F15" s="47" t="str">
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G15" s="47" t="str">
-        <x:v>Foundation uses one tool per play</x:v>
+        <x:v>Essentials uses one tool per play</x:v>
       </x:c>
       <x:c r="H15" s="50" t="str">
         <x:v>No</x:v>
@@ -1522,7 +1522,7 @@
         <x:v>Saved to My Account</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Saved to Foundation My Account after free registration</x:v>
+        <x:v>Saved to Essentials My Account after free registration</x:v>
       </x:c>
       <x:c r="F16" s="47" t="str">
         <x:v>Same</x:v>
@@ -1570,7 +1570,7 @@
         <x:v>Canonical shared maturity model template</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Same template/content with Foundation-local links</x:v>
+        <x:v>Same template/content with Essentials-local links</x:v>
       </x:c>
       <x:c r="F17" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -1624,13 +1624,13 @@
         <x:v>All 13 plays with full implementation guidance and related content</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>All 13 plays with appropriate public guidance and one Foundation Tool each</x:v>
+        <x:v>All 13 plays with appropriate public guidance and one Essentials Tool each</x:v>
       </x:c>
       <x:c r="F18" s="47" t="str">
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G18" s="47" t="str">
-        <x:v>Foundation limits protected facilitation methods and professional library depth</x:v>
+        <x:v>Essentials limits protected facilitation methods and professional library depth</x:v>
       </x:c>
       <x:c r="H18" s="50" t="str">
         <x:v>Review</x:v>
@@ -1768,13 +1768,13 @@
         <x:v>49 fillable tools</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>13 Foundation Tools, one per play</x:v>
+        <x:v>13 Essentials Tools, one per play</x:v>
       </x:c>
       <x:c r="F21" s="47" t="str">
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="G21" s="47" t="str">
-        <x:v>Foundation intentionally limits the professional tool library</x:v>
+        <x:v>Essentials intentionally limits the professional tool library</x:v>
       </x:c>
       <x:c r="H21" s="50" t="str">
         <x:v>No</x:v>
@@ -1822,7 +1822,7 @@
         <x:v>Checkboxes, dropdowns, repeatable Other values, text fields, dynamic documentation, compact RASCI, tasks</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Simpler Foundation fillable tool form</x:v>
+        <x:v>Simpler Essentials fillable tool form</x:v>
       </x:c>
       <x:c r="F22" s="47" t="str">
         <x:v>Limited</x:v>
@@ -1834,7 +1834,7 @@
         <x:v>Review</x:v>
       </x:c>
       <x:c r="I22" s="50" t="str">
-        <x:v>Document which guided controls are Foundation-appropriate without exposing protected methods</x:v>
+        <x:v>Document which guided controls are Essentials-appropriate without exposing protected methods</x:v>
       </x:c>
       <x:c r="J22" s="50" t="str">
         <x:v>High</x:v>
@@ -1876,7 +1876,7 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G23" s="47" t="str">
-        <x:v>Foundation guidance is shorter</x:v>
+        <x:v>Essentials guidance is shorter</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
         <x:v>Yes</x:v>
@@ -1918,7 +1918,7 @@
         <x:v>Scenario-based examples, hover guidance, and coherent examples across tool</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Foundation examples and instructions</x:v>
+        <x:v>Essentials examples and instructions</x:v>
       </x:c>
       <x:c r="F24" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -2014,7 +2014,7 @@
         <x:v>Download/print completed tools</x:v>
       </x:c>
       <x:c r="E26" s="47" t="str">
-        <x:v>Download/print Foundation Tools with free account</x:v>
+        <x:v>Download/print Essentials Tools with free account</x:v>
       </x:c>
       <x:c r="F26" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -2062,13 +2062,13 @@
         <x:v>89 developed modules across foundational, role-based, functional, leadership, and technical tracks</x:v>
       </x:c>
       <x:c r="E27" s="47" t="str">
-        <x:v>9 Foundation modules available; other developed modules described but not accessible</x:v>
+        <x:v>9 Essentials modules available; other developed modules described but not accessible</x:v>
       </x:c>
       <x:c r="F27" s="47" t="str">
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="G27" s="47" t="str">
-        <x:v>Foundation is an entry tier, not an unfinished curriculum</x:v>
+        <x:v>Essentials is an entry tier, not an unfinished curriculum</x:v>
       </x:c>
       <x:c r="H27" s="50" t="str">
         <x:v>Review</x:v>
@@ -2114,13 +2114,13 @@
         <x:v>Search, level, family, prerequisites, duration, and track sequencing</x:v>
       </x:c>
       <x:c r="E28" s="47" t="str">
-        <x:v>Foundation catalog and learning-track information</x:v>
+        <x:v>Essentials catalog and learning-track information</x:v>
       </x:c>
       <x:c r="F28" s="47" t="str">
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="G28" s="47" t="str">
-        <x:v>Foundation currently has fewer filtering needs</x:v>
+        <x:v>Essentials currently has fewer filtering needs</x:v>
       </x:c>
       <x:c r="H28" s="50" t="str">
         <x:v>Review</x:v>
@@ -2162,13 +2162,13 @@
         <x:v>All developed pathway modules available according to entitlement</x:v>
       </x:c>
       <x:c r="E29" s="47" t="str">
-        <x:v>Canned pathway information available; non-Foundation modules locked</x:v>
+        <x:v>Canned pathway information available; non-Essentials modules locked</x:v>
       </x:c>
       <x:c r="F29" s="47" t="str">
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G29" s="47" t="str">
-        <x:v>Foundation can view recommendations but not take locked modules</x:v>
+        <x:v>Essentials can view recommendations but not take locked modules</x:v>
       </x:c>
       <x:c r="H29" s="50" t="str">
         <x:v>No</x:v>
@@ -2258,13 +2258,13 @@
         <x:v>Tracks completed modules, assessment results, and recommendations</x:v>
       </x:c>
       <x:c r="E31" s="47" t="str">
-        <x:v>Tracks Foundation completions, assessment results, and recommendations</x:v>
+        <x:v>Tracks Essentials completions, assessment results, and recommendations</x:v>
       </x:c>
       <x:c r="F31" s="47" t="str">
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G31" s="47" t="str">
-        <x:v>Foundation cannot complete locked modules</x:v>
+        <x:v>Essentials cannot complete locked modules</x:v>
       </x:c>
       <x:c r="H31" s="50" t="str">
         <x:v>Yes</x:v>
@@ -2306,7 +2306,7 @@
         <x:v>Shared objectives, lessons, public health scenarios, practical application, knowledge check, references, related plays/tools</x:v>
       </x:c>
       <x:c r="E32" s="47" t="str">
-        <x:v>Same template for available Foundation modules; locked modules show edition availability</x:v>
+        <x:v>Same template for available Essentials modules; locked modules show edition availability</x:v>
       </x:c>
       <x:c r="F32" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -2354,13 +2354,13 @@
         <x:v>Administrator-oriented personal dashboard with saved work, learning, assessments, downloads, and tasks</x:v>
       </x:c>
       <x:c r="E33" s="47" t="str">
-        <x:v>Simple free-member account for downloads, assessment results, and Foundation learning</x:v>
+        <x:v>Simple free-member account for downloads, assessment results, and Essentials learning</x:v>
       </x:c>
       <x:c r="F33" s="47" t="str">
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G33" s="47" t="str">
-        <x:v>Foundation should be simpler and clearly individual</x:v>
+        <x:v>Essentials should be simpler and clearly individual</x:v>
       </x:c>
       <x:c r="H33" s="50" t="str">
         <x:v>Review</x:v>
@@ -2405,10 +2405,10 @@
         <x:v>Required for downloads, personalized learning assessment, and reviewer eligibility</x:v>
       </x:c>
       <x:c r="F34" s="47" t="str">
-        <x:v>Foundation Only</x:v>
+        <x:v>Essentials Only</x:v>
       </x:c>
       <x:c r="G34" s="47" t="str">
-        <x:v>Foundation membership is a trust and conversion mechanism</x:v>
+        <x:v>Essentials membership is a trust and conversion mechanism</x:v>
       </x:c>
       <x:c r="H34" s="50" t="str">
         <x:v>Yes</x:v>
@@ -2462,7 +2462,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I35" s="50" t="str">
-        <x:v>Keep navigation hidden in Foundation and describe benefit on edition pages</x:v>
+        <x:v>Keep navigation hidden in Essentials and describe benefit on edition pages</x:v>
       </x:c>
       <x:c r="J35" s="50" t="str">
         <x:v>High</x:v>
@@ -2552,7 +2552,7 @@
         <x:v>Limited</x:v>
       </x:c>
       <x:c r="G37" s="47" t="str">
-        <x:v>Foundation can build trust without releasing protected analysis</x:v>
+        <x:v>Essentials can build trust without releasing protected analysis</x:v>
       </x:c>
       <x:c r="H37" s="50" t="str">
         <x:v>Review</x:v>
@@ -2610,7 +2610,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I38" s="50" t="str">
-        <x:v>Use shared template and keep Foundation edition information outside Community</x:v>
+        <x:v>Use shared template and keep Essentials edition information outside Community</x:v>
       </x:c>
       <x:c r="J38" s="50" t="str">
         <x:v>Medium</x:v>
@@ -2652,7 +2652,7 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G39" s="47" t="str">
-        <x:v>Foundation emphasizes reviewer recruitment</x:v>
+        <x:v>Essentials emphasizes reviewer recruitment</x:v>
       </x:c>
       <x:c r="H39" s="50" t="str">
         <x:v>Yes</x:v>
@@ -2948,7 +2948,7 @@
         <x:v>Full contact route</x:v>
       </x:c>
       <x:c r="E45" s="47" t="str">
-        <x:v>Foundation contact route</x:v>
+        <x:v>Essentials contact route</x:v>
       </x:c>
       <x:c r="F45" s="47" t="str">
         <x:v>Same</x:v>
@@ -3002,7 +3002,7 @@
         <x:v>Adapted</x:v>
       </x:c>
       <x:c r="G46" s="47" t="str">
-        <x:v>Foundation release state must be independently tracked</x:v>
+        <x:v>Essentials release state must be independently tracked</x:v>
       </x:c>
       <x:c r="H46" s="50" t="str">
         <x:v>Yes</x:v>
@@ -3167,7 +3167,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="F5:F47">
-      <x:formula1>"Same,Adapted,Limited,Not Available,Foundation Only,Full Only,Needs Review"</x:formula1>
+      <x:formula1>"Same,Adapted,Limited,Not Available,Essentials Only,Full Only,Needs Review"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H5:H47">
       <x:formula1>"No,Yes,Review,TBD"</x:formula1>
@@ -3227,7 +3227,7 @@
         <x:v>Full Version Route</x:v>
       </x:c>
       <x:c r="D4" s="38" t="str">
-        <x:v>Foundation Route</x:v>
+        <x:v>Essentials Route</x:v>
       </x:c>
       <x:c r="E4" s="38" t="str">
         <x:v>Shared Template Type</x:v>
@@ -3236,7 +3236,7 @@
         <x:v>Full Content Scope</x:v>
       </x:c>
       <x:c r="G4" s="38" t="str">
-        <x:v>Foundation Content Scope</x:v>
+        <x:v>Essentials Content Scope</x:v>
       </x:c>
       <x:c r="H4" s="38" t="str">
         <x:v>Access Difference</x:v>
@@ -3280,7 +3280,7 @@
         <x:v>Full system overview and entry points</x:v>
       </x:c>
       <x:c r="G5" s="46" t="str">
-        <x:v>Foundation positioning, edition comparison, 13 plays/tools/modules</x:v>
+        <x:v>Essentials positioning, edition comparison, 13 plays/tools/modules</x:v>
       </x:c>
       <x:c r="H5" s="46" t="str">
         <x:v>Public in both</x:v>
@@ -3412,10 +3412,10 @@
         <x:v>Role-scaled questions and all recommendations</x:v>
       </x:c>
       <x:c r="G8" s="47" t="str">
-        <x:v>Same assessment; access labels reflect Foundation</x:v>
+        <x:v>Same assessment; access labels reflect Essentials</x:v>
       </x:c>
       <x:c r="H8" s="47" t="str">
-        <x:v>Free account required in Foundation</x:v>
+        <x:v>Free account required in Essentials</x:v>
       </x:c>
       <x:c r="I8" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -3456,7 +3456,7 @@
         <x:v>All entitled modules</x:v>
       </x:c>
       <x:c r="G9" s="47" t="str">
-        <x:v>Foundation modules; other editions unavailable</x:v>
+        <x:v>Essentials modules; other editions unavailable</x:v>
       </x:c>
       <x:c r="H9" s="47" t="str">
         <x:v>Entitlement differs</x:v>
@@ -3500,10 +3500,10 @@
         <x:v>Full recommendations and tools</x:v>
       </x:c>
       <x:c r="G10" s="47" t="str">
-        <x:v>Foundation recommendations and tools</x:v>
+        <x:v>Essentials recommendations and tools</x:v>
       </x:c>
       <x:c r="H10" s="47" t="str">
-        <x:v>Free account required in Foundation</x:v>
+        <x:v>Free account required in Essentials</x:v>
       </x:c>
       <x:c r="I10" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -3544,7 +3544,7 @@
         <x:v>Canonical model and links</x:v>
       </x:c>
       <x:c r="G11" s="47" t="str">
-        <x:v>Same model; Foundation-local links</x:v>
+        <x:v>Same model; Essentials-local links</x:v>
       </x:c>
       <x:c r="H11" s="47" t="str">
         <x:v>Public in both</x:v>
@@ -3632,7 +3632,7 @@
         <x:v>Complete relationships and implementation guidance</x:v>
       </x:c>
       <x:c r="G13" s="47" t="str">
-        <x:v>Public subset plus Foundation Tool</x:v>
+        <x:v>Public subset plus Essentials Tool</x:v>
       </x:c>
       <x:c r="H13" s="47" t="str">
         <x:v>Public in both</x:v>
@@ -3679,7 +3679,7 @@
         <x:v>13 tools</x:v>
       </x:c>
       <x:c r="H14" s="47" t="str">
-        <x:v>Foundation download requires account</x:v>
+        <x:v>Essentials download requires account</x:v>
       </x:c>
       <x:c r="I14" s="47" t="str">
         <x:v>Limited</x:v>
@@ -3720,7 +3720,7 @@
         <x:v>Advanced guided Full tool</x:v>
       </x:c>
       <x:c r="G15" s="47" t="str">
-        <x:v>Simpler Foundation Tool</x:v>
+        <x:v>Simpler Essentials Tool</x:v>
       </x:c>
       <x:c r="H15" s="47" t="str">
         <x:v>Entitlement and depth differ</x:v>
@@ -3811,7 +3811,7 @@
         <x:v>Simple free-member dashboard</x:v>
       </x:c>
       <x:c r="H17" s="47" t="str">
-        <x:v>Foundation is individual-only</x:v>
+        <x:v>Essentials is individual-only</x:v>
       </x:c>
       <x:c r="I17" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -3943,7 +3943,7 @@
         <x:v>Same; free account prerequisite for reviewers</x:v>
       </x:c>
       <x:c r="H20" s="47" t="str">
-        <x:v>Foundation membership differs</x:v>
+        <x:v>Essentials membership differs</x:v>
       </x:c>
       <x:c r="I20" s="47" t="str">
         <x:v>Adapted</x:v>
@@ -4366,7 +4366,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Stable IDs for plays, tools, and the Foundation learning subset. The canonical Full catalog remains the source of truth for all detailed module records.</x:v>
+        <x:v>Stable IDs for plays, tools, and the Essentials learning subset. The canonical Full catalog remains the source of truth for all detailed module records.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -4386,10 +4386,10 @@
         <x:v>Full Version Availability</x:v>
       </x:c>
       <x:c r="F4" s="38" t="str">
-        <x:v>Foundation Availability</x:v>
+        <x:v>Essentials Availability</x:v>
       </x:c>
       <x:c r="G4" s="38" t="str">
-        <x:v>Foundation Mapping / Notes</x:v>
+        <x:v>Essentials Mapping / Notes</x:v>
       </x:c>
       <x:c r="H4" s="38" t="str">
         <x:v>Target / Release Version</x:v>
@@ -4753,7 +4753,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G18" s="50" t="str">
-        <x:v>Foundation Tool for Play 1</x:v>
+        <x:v>Essentials Tool for Play 1</x:v>
       </x:c>
       <x:c r="H18" s="56" t="str">
         <x:v>0.9</x:v>
@@ -4909,7 +4909,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Foundation Tool for Play 2</x:v>
+        <x:v>Essentials Tool for Play 2</x:v>
       </x:c>
       <x:c r="H24" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5013,7 +5013,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G28" s="50" t="str">
-        <x:v>Foundation Tool for Play 3</x:v>
+        <x:v>Essentials Tool for Play 3</x:v>
       </x:c>
       <x:c r="H28" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5273,7 +5273,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G38" s="50" t="str">
-        <x:v>Foundation Tool for Play 4</x:v>
+        <x:v>Essentials Tool for Play 4</x:v>
       </x:c>
       <x:c r="H38" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5377,7 +5377,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G42" s="50" t="str">
-        <x:v>Foundation Tool for Play 5</x:v>
+        <x:v>Essentials Tool for Play 5</x:v>
       </x:c>
       <x:c r="H42" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5481,7 +5481,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G46" s="50" t="str">
-        <x:v>Foundation Tool for Play 10</x:v>
+        <x:v>Essentials Tool for Play 10</x:v>
       </x:c>
       <x:c r="H46" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5507,7 +5507,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G47" s="50" t="str">
-        <x:v>Foundation Tool for Play 6</x:v>
+        <x:v>Essentials Tool for Play 6</x:v>
       </x:c>
       <x:c r="H47" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5663,7 +5663,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G53" s="50" t="str">
-        <x:v>Foundation Tool for Play 9</x:v>
+        <x:v>Essentials Tool for Play 9</x:v>
       </x:c>
       <x:c r="H53" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5897,7 +5897,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G62" s="50" t="str">
-        <x:v>Foundation Tool for Play 13</x:v>
+        <x:v>Essentials Tool for Play 13</x:v>
       </x:c>
       <x:c r="H62" s="56" t="str">
         <x:v>0.9</x:v>
@@ -5923,7 +5923,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G63" s="50" t="str">
-        <x:v>Foundation Tool for Play 12</x:v>
+        <x:v>Essentials Tool for Play 12</x:v>
       </x:c>
       <x:c r="H63" s="56" t="str">
         <x:v>0.9</x:v>
@@ -6053,7 +6053,7 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="G68" s="50" t="str">
-        <x:v>Foundation module</x:v>
+        <x:v>Essentials module</x:v>
       </x:c>
       <x:c r="H68" s="56" t="str">
         <x:v>0.9</x:v>
@@ -6358,7 +6358,7 @@
         <x:v>PLAT-002</x:v>
       </x:c>
       <x:c r="C5" s="49" t="str">
-        <x:v>Use the same page templates across Full and Foundation editions</x:v>
+        <x:v>Use the same page templates across Full and Essentials editions</x:v>
       </x:c>
       <x:c r="D5" s="49" t="str">
         <x:v>Product consistency decision</x:v>
@@ -6396,7 +6396,7 @@
         <x:v>HOME-004</x:v>
       </x:c>
       <x:c r="C6" s="50" t="str">
-        <x:v>Differentiate Foundation free/low-cost release from forthcoming robust editions</x:v>
+        <x:v>Differentiate Essentials free/low-cost release from forthcoming robust editions</x:v>
       </x:c>
       <x:c r="D6" s="50" t="str">
         <x:v>Homepage positioning review</x:v>
@@ -6423,7 +6423,7 @@
         <x:v>17dea89</x:v>
       </x:c>
       <x:c r="L6" s="50" t="str">
-        <x:v>Foundation edition comparison and concise overview released</x:v>
+        <x:v>Essentials edition comparison and concise overview released</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -6434,7 +6434,7 @@
         <x:v>GOV-001</x:v>
       </x:c>
       <x:c r="C7" s="51" t="str">
-        <x:v>Create Full/Foundation edition crosswalk for version control and future updates</x:v>
+        <x:v>Create Full/Essentials edition crosswalk for version control and future updates</x:v>
       </x:c>
       <x:c r="D7" s="51" t="str">
         <x:v>Product governance request</x:v>
@@ -7995,7 +7995,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="C6" s="35" t="str">
-        <x:v>Same; Adapted; Limited; Not Available; Foundation Only; Full Only; Needs Review</x:v>
+        <x:v>Same; Adapted; Limited; Not Available; Essentials Only; Full Only; Needs Review</x:v>
       </x:c>
       <x:c r="D6" s="35" t="str">
         <x:v>Relationship between editions</x:v>
@@ -8129,7 +8129,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="35" t="str">
-        <x:v>Full / Foundation Route</x:v>
+        <x:v>Full / Essentials Route</x:v>
       </x:c>
       <x:c r="B13" s="35" t="str">
         <x:v>When applicable</x:v>
@@ -8141,7 +8141,7 @@
         <x:v>Edition-local destination or source</x:v>
       </x:c>
       <x:c r="E13" s="35" t="str">
-        <x:v>Never point a Foundation user into Full unless explicitly labeled</x:v>
+        <x:v>Never point a Essentials user into Full unless explicitly labeled</x:v>
       </x:c>
       <x:c r="F13" s="35" t="str">
         <x:v>Prefer route helpers over hardcoded URLs</x:v>
@@ -8195,7 +8195,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="C16" s="36" t="str">
-        <x:v>Foundation 0.9 → Foundation 1.0; Organization 1.0; Enterprise 1.0</x:v>
+        <x:v>Essentials 0.9 → Essentials 1.0; Organization 1.0; Enterprise 1.0</x:v>
       </x:c>
       <x:c r="D16" s="36" t="str">
         <x:v>Product release naming convention</x:v>

</xml_diff>